<commit_message>
docs: add cybersecurity audit report and security tracking spreadsheets
</commit_message>
<xml_diff>
--- a/Pentest-Security-Report.xlsx
+++ b/Pentest-Security-Report.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Pentest Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Security Measures" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +77,14 @@
       <color rgb="007F6000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00843C0B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +131,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -151,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -187,6 +199,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1659,4 +1674,614 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MyPLC - Security Measures (what protects the app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>As of 2026-10-28  -  25 measures:  21 in place,  0 partial,  4 to add.  The security logic that protects MyPLC. (The 'Pentest Report' tab has the test results that back these up.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>What it does (plain)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>How it's done in MyPLC</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Memory-safe code</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Prevents whole classes of hacking bugs (buffer overflows, memory corruption).</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Backend written in Rust with zero 'unsafe' code.</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Login / token on the network</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Only someone with the right key can connect and control the PLC.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>A network address is refused without a token; every connection is checked.</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Brute-force lockout</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Stops password guessing by many fast attempts.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>After 5 wrong tokens the attacker's machine is locked out, 1s pause per try.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Big-message limit</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>One huge message can't exhaust memory / crash the server.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Messages and frames capped at 1 MB.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Connection limit</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>A flood of connections can't overwhelm the server.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Capped at 128 simultaneous connections.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Input validation</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Broken or hostile messages are rejected cleanly.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Strict JSON decoding; bad input gets a 'rejected' reply and the server stays up.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>SQL-injection safe</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Attackers can't inject database commands.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>All database queries are fixed; user text is never pasted into SQL.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Path-traversal block</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Tricks like '../../' can't reach files outside the project.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>File paths are validated; anything escaping the project folder is rejected.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Runaway-program limits</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>A bad PLC program (endless loop, giant arrays) can't freeze the system.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Loop cap 100,000/scan; array and nesting limits; stops safely on a scan error.</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Safe error messages</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Error text doesn't leak secrets (paths, versions).</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Users see friendly messages; technical detail goes only to the server log.</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Security header (nosniff)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Stops the browser guessing content types (an attack vector).</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>X-Content-Type-Options: nosniff on the server's web replies.</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Content Security Policy (CSP)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Blocks injected/malicious scripts in the desktop app.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>A strict CSP allowing only what the app and editor need.</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>SCADA value checks</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Bad tag values (NaN, infinity, wrong type) can't poison the system.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Non-finite and wrong-typed values are rejected before use.</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Secrets kept out of code</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>No passwords/keys hardcoded in the source.</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>All secrets read from environment settings; .env is git-ignored and never committed.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Secrets kept out of logs</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Tokens/passwords never written to log files.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Logs record who connected, never the token value.</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dependency scanning</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Catches known security holes in third-party libraries.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>cargo audit + npm audit run and all findings fixed; now clean.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Encryption in transit (TLS)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Scrambles data on the wire so it can't be read or altered.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Render provides HTTPS/WSS on the public link (edge TLS). Internal links are on a trusted network.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Live monitoring</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>See the system's health and connected devices in real time.</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Prometheus /metrics endpoint (token-protected) + Grafana dashboard.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Auto-recovery after restart</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>The PLC comes back in the same state after a crash/reboot.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>The loaded project and RUN/STOP mode are saved and restored on startup.</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Crash isolation</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>One part failing shouldn't take the whole server down.</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Each client on its own thread; the shared lock recovers from a poisoned state; scans are wrapped so an unexpected crash stops the PLC cleanly instead of freezing.</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Per-user login &amp; roles (RBAC)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Know WHO did what; limit who can Start/Stop vs view.</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Not built yet - one shared token today. Needed before multiple users or remote access.</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>To add</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Keep the token out of the installer</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>The shared app shouldn't contain the backend password.</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Done - the token is entered on first launch and stored on the user's machine (Settings &gt; Backend), not built into the app. The shared installer has no secret.</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>In place</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Installer code signing</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Proves the app is genuine and untampered.</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>The installer is unsigned - sign it before wide distribution.</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>To add</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SCADA source authentication</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Make sure tag values come from the real SCADA, not a fake.</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>The backend trusts its configured SCADA source (rejects garbage). True source auth is a SCADA-side control.</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>To add</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Firewall / database exposure check</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Keep the database and ports off the open internet.</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>A deployment step to verify - make sure DB port 5432 isn't world-reachable.</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>To add</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>